<commit_message>
Update dashboard and report presentation
</commit_message>
<xml_diff>
--- a/DATA/UGSN_INFO.xlsx
+++ b/DATA/UGSN_INFO.xlsx
@@ -2566,8 +2566,12 @@
       <c r="A7" s="70" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="48"/>
-      <c r="C7" s="50"/>
+      <c r="B7" s="48">
+        <v>152</v>
+      </c>
+      <c r="C7" s="50">
+        <v>20</v>
+      </c>
       <c r="D7" s="48"/>
       <c r="E7" s="50"/>
       <c r="F7" s="71"/>

</xml_diff>